<commit_message>
Renaming main control file
</commit_message>
<xml_diff>
--- a/Master_Control_File.xlsx
+++ b/Master_Control_File.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aprashar\Documents\Github\DWRAT_DataScraping\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D83BC658-7AF7-469C-849F-A5DC75E2FB66}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C936A5A-DA08-4724-A281-9167EB21B498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
   <si>
     <t>VALUE</t>
   </si>
@@ -109,9 +109,6 @@
   </si>
   <si>
     <t>URL that points to "My Content" on ArcGIS Portal</t>
-  </si>
-  <si>
-    <t>TEST</t>
   </si>
 </sst>
 </file>
@@ -440,7 +437,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
@@ -585,11 +582,6 @@
         <v>27</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="B13" t="s">
-        <v>28</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updating file to create a merge conflict
Need screenshots for a tutorial
</commit_message>
<xml_diff>
--- a/Master_Control_File.xlsx
+++ b/Master_Control_File.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aprashar\Documents\Github\DWRAT_DataScraping\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aprashar\Pictures\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C936A5A-DA08-4724-A281-9167EB21B498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB9095C6-52D4-4B2B-B3F3-1C1785D4408A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
   <si>
     <t>VALUE</t>
   </si>
@@ -109,6 +109,15 @@
   </si>
   <si>
     <t>URL that points to "My Content" on ArcGIS Portal</t>
+  </si>
+  <si>
+    <t>TEST</t>
+  </si>
+  <si>
+    <t>TEST_ROW</t>
+  </si>
+  <si>
+    <t>Getting screenshots for a tutorial on resolving conflicts</t>
   </si>
 </sst>
 </file>
@@ -437,16 +446,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="62.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="62.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -460,7 +469,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -471,7 +480,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -482,7 +491,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -493,7 +502,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -504,7 +513,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -515,7 +524,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -526,7 +535,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -537,7 +546,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -548,7 +557,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -559,7 +568,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -570,7 +579,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -580,6 +589,17 @@
       <c r="C12" s="1"/>
       <c r="D12" t="s">
         <v>27</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>28</v>
+      </c>
+      <c r="B13" t="s">
+        <v>29</v>
+      </c>
+      <c r="D13" t="s">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Resetting control file after messing with it
</commit_message>
<xml_diff>
--- a/Master_Control_File.xlsx
+++ b/Master_Control_File.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aprashar\Pictures\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aprashar\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB9095C6-52D4-4B2B-B3F3-1C1785D4408A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5861D31E-E116-4774-AF00-A0063E881825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2268" yWindow="2268" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
   <si>
     <t>VALUE</t>
   </si>
@@ -109,15 +109,6 @@
   </si>
   <si>
     <t>URL that points to "My Content" on ArcGIS Portal</t>
-  </si>
-  <si>
-    <t>TEST</t>
-  </si>
-  <si>
-    <t>TEST_ROW</t>
-  </si>
-  <si>
-    <t>Getting screenshots for a tutorial on resolving conflicts</t>
   </si>
 </sst>
 </file>
@@ -446,16 +437,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D12"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.7109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="62.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="62.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>4</v>
       </c>
@@ -469,7 +460,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -480,7 +471,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -491,7 +482,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -502,7 +493,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -513,7 +504,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -524,7 +515,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -535,7 +526,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>5</v>
       </c>
@@ -546,7 +537,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>5</v>
       </c>
@@ -557,7 +548,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>5</v>
       </c>
@@ -568,7 +559,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>5</v>
       </c>
@@ -579,7 +570,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -589,17 +580,6 @@
       <c r="C12" s="1"/>
       <c r="D12" t="s">
         <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" t="s">
-        <v>29</v>
-      </c>
-      <c r="D13" t="s">
-        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Deleted generic Paradigm DWRAT repo
</commit_message>
<xml_diff>
--- a/Master_Control_File.xlsx
+++ b/Master_Control_File.xlsx
@@ -1,31 +1,48 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aprashar\Documents\Github\DWRAT_DataScraping\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cawaterboards.sharepoint.com/DWR/SDA/Shared Documents/Program Watersheds/4. Demand Data Tracking/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C936A5A-DA08-4724-A281-9167EB21B498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="13_ncr:1_{2C936A5A-DA08-4724-A281-9167EB21B498}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E664978A-C1E3-4E3B-A8B4-E5D6FE4E7907}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11904" yWindow="12852" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="44">
+  <si>
+    <t>CATEGORY</t>
+  </si>
+  <si>
+    <t>FIELD</t>
+  </si>
   <si>
     <t>VALUE</t>
   </si>
@@ -33,18 +50,12 @@
     <t>DESCRIPTION</t>
   </si>
   <si>
-    <t>FIELD</t>
+    <t>DEMAND</t>
   </si>
   <si>
     <t>FLAT_FILE_DATABASE_SERVER</t>
   </si>
   <si>
-    <t>CATEGORY</t>
-  </si>
-  <si>
-    <t>DEMAND</t>
-  </si>
-  <si>
     <t>Database server name</t>
   </si>
   <si>
@@ -66,24 +77,24 @@
     <t>Table information for the primary eWRIMS flat file</t>
   </si>
   <si>
+    <t>FLAT_FILE_REPORTING_TABLE_NAME</t>
+  </si>
+  <si>
     <t>Table information for the eWRIMS reporting flat file</t>
   </si>
   <si>
-    <t>FLAT_FILE_REPORTING_TABLE_NAME</t>
-  </si>
-  <si>
     <t>FLAT_FILE_EXTENDED_REPORTING_TABLE_NAME</t>
   </si>
   <si>
     <t>Table information for the extended eWRIMS reporting flat file</t>
   </si>
   <si>
+    <t>FLAT_FILE_USE_SEASON_TABLE_NAME</t>
+  </si>
+  <si>
     <t>Table information for the eWRIMS use season flat file</t>
   </si>
   <si>
-    <t>FLAT_FILE_USE_SEASON_TABLE_NAME</t>
-  </si>
-  <si>
     <t>FLAT_FILE_PARTY_TABLE_NAME</t>
   </si>
   <si>
@@ -96,9 +107,6 @@
     <t>The location of SharePoint folders synced locally by OneDrive</t>
   </si>
   <si>
-    <t>The SharePoint version of "Watershed_Demand_Dataset_Paths.xlsx"</t>
-  </si>
-  <si>
     <t>SHAREPOINT_DEMAND_CONTROL_FILE</t>
   </si>
   <si>
@@ -109,6 +117,57 @@
   </si>
   <si>
     <t>URL that points to "My Content" on ArcGIS Portal</t>
+  </si>
+  <si>
+    <t>ReportDB</t>
+  </si>
+  <si>
+    <t>reportmanager,1542</t>
+  </si>
+  <si>
+    <t>ReportDB.FLAT_FILE.ewrims_flat_file_pod</t>
+  </si>
+  <si>
+    <t>ReportDB.FLAT_FILE.ewrims_flat_file</t>
+  </si>
+  <si>
+    <t>ReportDB.FLAT_FILE.ewrims_water_use_report</t>
+  </si>
+  <si>
+    <t>ReportDB.FLAT_FILE.ewrims_water_use_report_extended</t>
+  </si>
+  <si>
+    <t>ReportDB.FLAT_FILE.ewrims_flat_file_use_season</t>
+  </si>
+  <si>
+    <t>ReportDB.FLAT_FILE.ewrims_flat_file_party</t>
+  </si>
+  <si>
+    <t>GENERAL</t>
+  </si>
+  <si>
+    <t>Water Boards/Supply and Demand Assessment - Documents/</t>
+  </si>
+  <si>
+    <t>Program Watersheds/4. Demand Data Tracking/Watershed_Demand_Dataset_Paths.xlsx</t>
+  </si>
+  <si>
+    <t>Partial path to the SharePoint version of "Watershed_Demand_Dataset_Paths.xlsx"</t>
+  </si>
+  <si>
+    <t>https://gispublic.waterboards.ca.gov/portal/home/content.html#my</t>
+  </si>
+  <si>
+    <t>RR_WORKFLOW</t>
+  </si>
+  <si>
+    <t>SHAREPOINT_RR_WORKFLOW_CONTROL_FILE</t>
+  </si>
+  <si>
+    <t>DWRAT\SDU_Runs\Automated_Procedure\RR_Workflow\RR_Workflow_Control_File.xlsx</t>
+  </si>
+  <si>
+    <t>Partial path to the SharePoint version of "RR_Workflow_Control_File.xlsx"</t>
   </si>
 </sst>
 </file>
@@ -132,12 +191,36 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0070C0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC00000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -153,15 +236,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -172,6 +274,19 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{1E9A3D38-4FF1-4DC9-8FA7-63E1C5E19866}" name="Table1" displayName="Table1" ref="A1:D13" totalsRowShown="0">
+  <autoFilter ref="A1:D13" xr:uid="{1E9A3D38-4FF1-4DC9-8FA7-63E1C5E19866}"/>
+  <tableColumns count="4">
+    <tableColumn id="1" xr3:uid="{3D1034EE-0DF5-48BB-B876-A05F139AC539}" name="CATEGORY" dataDxfId="0"/>
+    <tableColumn id="2" xr3:uid="{D4B26CB1-18FC-4911-8712-C55EB077B0EE}" name="FIELD"/>
+    <tableColumn id="3" xr3:uid="{868F6D54-9C0F-4924-B940-856230315B15}" name="VALUE"/>
+    <tableColumn id="4" xr3:uid="{71318BDA-7E76-40C7-BA73-AC6D359DF983}" name="DESCRIPTION"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium15" showFirstColumn="1" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -437,152 +552,509 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.88671875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="62.109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="50.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="62.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B1" t="s">
-        <v>2</v>
-      </c>
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
-      <c r="D1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="B2" t="s">
-        <v>3</v>
+      <c r="C2" t="s">
+        <v>28</v>
       </c>
       <c r="D2" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="B3" t="s">
         <v>7</v>
       </c>
+      <c r="C3" t="s">
+        <v>27</v>
+      </c>
       <c r="D3" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>5</v>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="B4" t="s">
         <v>9</v>
       </c>
+      <c r="C4" t="s">
+        <v>29</v>
+      </c>
       <c r="D4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
-        <v>5</v>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="B5" t="s">
         <v>11</v>
       </c>
+      <c r="C5" t="s">
+        <v>30</v>
+      </c>
       <c r="D5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>5</v>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="B6" t="s">
+        <v>13</v>
+      </c>
+      <c r="C6" t="s">
+        <v>31</v>
+      </c>
+      <c r="D6" t="s">
         <v>14</v>
       </c>
-      <c r="D6" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>5</v>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="B7" t="s">
         <v>15</v>
       </c>
+      <c r="C7" t="s">
+        <v>32</v>
+      </c>
       <c r="D7" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>5</v>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="B8" t="s">
+        <v>17</v>
+      </c>
+      <c r="C8" t="s">
+        <v>33</v>
+      </c>
+      <c r="D8" t="s">
         <v>18</v>
       </c>
-      <c r="D8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
-        <v>5</v>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="B9" t="s">
         <v>19</v>
       </c>
+      <c r="C9" t="s">
+        <v>34</v>
+      </c>
       <c r="D9" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
-        <v>5</v>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="3" t="s">
+        <v>35</v>
       </c>
       <c r="B10" t="s">
         <v>21</v>
       </c>
+      <c r="C10" t="s">
+        <v>36</v>
+      </c>
       <c r="D10" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
-        <v>5</v>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>4</v>
       </c>
       <c r="B11" t="s">
+        <v>23</v>
+      </c>
+      <c r="C11" t="s">
+        <v>37</v>
+      </c>
+      <c r="D11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D11" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="B12" t="s">
         <v>25</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D12" t="s">
         <v>26</v>
       </c>
-      <c r="C12" s="1"/>
-      <c r="D12" t="s">
-        <v>27</v>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="B13" t="s">
+        <v>41</v>
+      </c>
+      <c r="C13" t="s">
+        <v>42</v>
+      </c>
+      <c r="D13" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="C12" r:id="rId1" location="my" xr:uid="{C031276D-7092-433D-AE9B-C0770156E297}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
+</file>
+
+<file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="b2cf8adb-cf25-47fc-8c92-b53f2a7e7f06">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="851dfaa3-aae8-4c03-b90c-7dd4a6526d0d" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100F312EB754F236045A0D3EDD082CC91AE" ma:contentTypeVersion="16" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="e3883cbc254ec137d27422a2b14befbf">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="b2cf8adb-cf25-47fc-8c92-b53f2a7e7f06" xmlns:ns3="851dfaa3-aae8-4c03-b90c-7dd4a6526d0d" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="1be2573fe1476a916a702a25e6de1105" ns2:_="" ns3:_="">
+    <xsd:import namespace="b2cf8adb-cf25-47fc-8c92-b53f2a7e7f06"/>
+    <xsd:import namespace="851dfaa3-aae8-4c03-b90c-7dd4a6526d0d"/>
+    <xsd:element name="properties">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element name="documentManagement">
+            <xsd:complexType>
+              <xsd:all>
+                <xsd:element ref="ns2:MediaServiceMetadata" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceFastMetadata" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithUsers" minOccurs="0"/>
+                <xsd:element ref="ns3:SharedWithDetails" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceDateTaken" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaLengthInSeconds" minOccurs="0"/>
+                <xsd:element ref="ns2:lcf76f155ced4ddcb4097134ff3c332f" minOccurs="0"/>
+                <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceOCR" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceGenerationTime" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceEventHashCode" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceLocation" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
+              </xsd:all>
+            </xsd:complexType>
+          </xsd:element>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="b2cf8adb-cf25-47fc-8c92-b53f2a7e7f06" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="MediaServiceMetadata" ma:index="8" nillable="true" ma:displayName="MediaServiceMetadata" ma:hidden="true" ma:internalName="MediaServiceMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceFastMetadata" ma:index="9" nillable="true" ma:displayName="MediaServiceFastMetadata" ma:hidden="true" ma:internalName="MediaServiceFastMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceDateTaken" ma:index="12" nillable="true" ma:displayName="MediaServiceDateTaken" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceDateTaken" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaLengthInSeconds" ma:index="13" nillable="true" ma:displayName="MediaLengthInSeconds" ma:hidden="true" ma:internalName="MediaLengthInSeconds" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Unknown"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="15" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="1cfdcae8-6a83-4c52-b891-75b08cbe23e4" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+      <xsd:complexType>
+        <xsd:sequence>
+          <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
+        </xsd:sequence>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="MediaServiceOCR" ma:index="17" nillable="true" ma:displayName="Extracted Text" ma:internalName="MediaServiceOCR" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceGenerationTime" ma:index="18" nillable="true" ma:displayName="MediaServiceGenerationTime" ma:hidden="true" ma:internalName="MediaServiceGenerationTime" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceEventHashCode" ma:index="19" nillable="true" ma:displayName="MediaServiceEventHashCode" ma:hidden="true" ma:internalName="MediaServiceEventHashCode" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="20" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceLocation" ma:index="21" nillable="true" ma:displayName="Location" ma:indexed="true" ma:internalName="MediaServiceLocation" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceSearchProperties" ma:index="22" nillable="true" ma:displayName="MediaServiceSearchProperties" ma:hidden="true" ma:internalName="MediaServiceSearchProperties" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="23" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
+      </xsd:simpleType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="851dfaa3-aae8-4c03-b90c-7dd4a6526d0d" elementFormDefault="qualified">
+    <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <xsd:element name="SharedWithUsers" ma:index="10" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:UserMulti">
+            <xsd:sequence>
+              <xsd:element name="UserInfo" minOccurs="0" maxOccurs="unbounded">
+                <xsd:complexType>
+                  <xsd:sequence>
+                    <xsd:element name="DisplayName" type="xsd:string" minOccurs="0"/>
+                    <xsd:element name="AccountId" type="dms:UserId" minOccurs="0" nillable="true"/>
+                    <xsd:element name="AccountType" type="xsd:string" minOccurs="0"/>
+                  </xsd:sequence>
+                </xsd:complexType>
+              </xsd:element>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+    <xsd:element name="SharedWithDetails" ma:index="11" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note">
+          <xsd:maxLength value="255"/>
+        </xsd:restriction>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="TaxCatchAll" ma:index="16" nillable="true" ma:displayName="Taxonomy Catch All Column" ma:hidden="true" ma:list="{3bde447f-9c6c-4421-af29-e30b317a6074}" ma:internalName="TaxCatchAll" ma:showField="CatchAllData" ma:web="851dfaa3-aae8-4c03-b90c-7dd4a6526d0d">
+      <xsd:complexType>
+        <xsd:complexContent>
+          <xsd:extension base="dms:MultiChoiceLookup">
+            <xsd:sequence>
+              <xsd:element name="Value" type="dms:Lookup" maxOccurs="unbounded" minOccurs="0" nillable="true"/>
+            </xsd:sequence>
+          </xsd:extension>
+        </xsd:complexContent>
+      </xsd:complexType>
+    </xsd:element>
+  </xsd:schema>
+  <xsd:schema xmlns="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:odoc="http://schemas.microsoft.com/internal/obd" targetNamespace="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" elementFormDefault="qualified" attributeFormDefault="unqualified" blockDefault="#all">
+    <xsd:import namespace="http://purl.org/dc/elements/1.1/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dc.xsd"/>
+    <xsd:import namespace="http://purl.org/dc/terms/" schemaLocation="http://dublincore.org/schemas/xmls/qdc/2003/04/02/dcterms.xsd"/>
+    <xsd:element name="coreProperties" type="CT_coreProperties"/>
+    <xsd:complexType name="CT_coreProperties">
+      <xsd:all>
+        <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
+        <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dc:language" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="category" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="version" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element name="revision" minOccurs="0" maxOccurs="1" type="xsd:string">
+          <xsd:annotation>
+            <xsd:documentation>
+                        This value indicates the number of saves or revisions. The application is responsible for updating this value after each revision.
+                    </xsd:documentation>
+          </xsd:annotation>
+        </xsd:element>
+        <xsd:element name="lastModifiedBy" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+        <xsd:element ref="dcterms:modified" minOccurs="0" maxOccurs="1"/>
+        <xsd:element name="contentStatus" minOccurs="0" maxOccurs="1" type="xsd:string"/>
+      </xsd:all>
+    </xsd:complexType>
+  </xsd:schema>
+  <xs:schema xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" xmlns:xs="http://www.w3.org/2001/XMLSchema" targetNamespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" elementFormDefault="qualified" attributeFormDefault="unqualified">
+    <xs:element name="Person">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:DisplayName" minOccurs="0"/>
+          <xs:element ref="pc:AccountId" minOccurs="0"/>
+          <xs:element ref="pc:AccountType" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="DisplayName" type="xs:string"/>
+    <xs:element name="AccountId" type="xs:string"/>
+    <xs:element name="AccountType" type="xs:string"/>
+    <xs:element name="BDCAssociatedEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:BDCEntity" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+        <xs:attribute ref="pc:EntityNamespace"/>
+        <xs:attribute ref="pc:EntityName"/>
+        <xs:attribute ref="pc:SystemInstanceName"/>
+        <xs:attribute ref="pc:AssociationName"/>
+      </xs:complexType>
+    </xs:element>
+    <xs:attribute name="EntityNamespace" type="xs:string"/>
+    <xs:attribute name="EntityName" type="xs:string"/>
+    <xs:attribute name="SystemInstanceName" type="xs:string"/>
+    <xs:attribute name="AssociationName" type="xs:string"/>
+    <xs:element name="BDCEntity">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:EntityDisplayName" minOccurs="0"/>
+          <xs:element ref="pc:EntityInstanceReference" minOccurs="0"/>
+          <xs:element ref="pc:EntityId1" minOccurs="0"/>
+          <xs:element ref="pc:EntityId2" minOccurs="0"/>
+          <xs:element ref="pc:EntityId3" minOccurs="0"/>
+          <xs:element ref="pc:EntityId4" minOccurs="0"/>
+          <xs:element ref="pc:EntityId5" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="EntityDisplayName" type="xs:string"/>
+    <xs:element name="EntityInstanceReference" type="xs:string"/>
+    <xs:element name="EntityId1" type="xs:string"/>
+    <xs:element name="EntityId2" type="xs:string"/>
+    <xs:element name="EntityId3" type="xs:string"/>
+    <xs:element name="EntityId4" type="xs:string"/>
+    <xs:element name="EntityId5" type="xs:string"/>
+    <xs:element name="Terms">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermInfo" minOccurs="0" maxOccurs="unbounded"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermInfo">
+      <xs:complexType>
+        <xs:sequence>
+          <xs:element ref="pc:TermName" minOccurs="0"/>
+          <xs:element ref="pc:TermId" minOccurs="0"/>
+        </xs:sequence>
+      </xs:complexType>
+    </xs:element>
+    <xs:element name="TermName" type="xs:string"/>
+    <xs:element name="TermId" type="xs:string"/>
+  </xs:schema>
+</ct:contentTypeSchema>
+</file>
+
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C777B51-B781-4DFC-B275-17C4099AC1EE}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="b2cf8adb-cf25-47fc-8c92-b53f2a7e7f06"/>
+    <ds:schemaRef ds:uri="851dfaa3-aae8-4c03-b90c-7dd4a6526d0d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2142662B-DCFE-4720-A631-17ADFCB1740E}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{75EF67B1-507D-41EA-B811-F716B8AE4334}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="b2cf8adb-cf25-47fc-8c92-b53f2a7e7f06"/>
+    <ds:schemaRef ds:uri="851dfaa3-aae8-4c03-b90c-7dd4a6526d0d"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=docMetadata/LabelInfo.xml><?xml version="1.0" encoding="utf-8"?>
+<clbl:labelList xmlns:clbl="http://schemas.microsoft.com/office/2020/mipLabelMetadata">
+  <clbl:label id="{0bb6ca0c-ccb3-428b-9d5f-a9c60cad6645}" enabled="1" method="Standard" siteId="{fe186a25-7d49-41e6-9941-05d2281d36c1}" removed="0"/>
+</clbl:labelList>
 </file>
</xml_diff>